<commit_message>
made changes in User and Url, ProjectWebServices
</commit_message>
<xml_diff>
--- a/src/main/resources/ProgressReport_Field_Values.xlsx
+++ b/src/main/resources/ProgressReport_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Product Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Product\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB70D57A-12DA-4020-A28A-A55205612796}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96317787-37C9-421F-A0DC-043CD533A2BE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="11" activeTab="16" xr2:uid="{2CF227FB-55E5-4154-93E7-6831A7625F64}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="9" activeTab="11" xr2:uid="{2CF227FB-55E5-4154-93E7-6831A7625F64}"/>
   </bookViews>
   <sheets>
     <sheet name="Edition" sheetId="1" r:id="rId1"/>
@@ -36,17 +36,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="82">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -102,12 +97,6 @@
     <t>the major changes in the organization’s capacity over the past year that have impacted or may impact the progress of the funded project, including changes</t>
   </si>
   <si>
-    <t>PatientPopulationTarget__c</t>
-  </si>
-  <si>
-    <t>NoOfPatientsServedInQuarter__c</t>
-  </si>
-  <si>
     <t>GoverningOrganizationReportDate__c</t>
   </si>
   <si>
@@ -280,6 +269,24 @@
   </si>
   <si>
     <t>Automation award for PR</t>
+  </si>
+  <si>
+    <t>fieldProjectNarrative__c</t>
+  </si>
+  <si>
+    <t>fieldOrganizationalCapacity__c</t>
+  </si>
+  <si>
+    <t>fieldPatientPopulationTarget__c</t>
+  </si>
+  <si>
+    <t>fieldNoOfPatientsServedInQuarter__c</t>
+  </si>
+  <si>
+    <t>fieldGoverningOrganizationReportDate__c</t>
+  </si>
+  <si>
+    <t>fieldBoardInformation__c</t>
   </si>
 </sst>
 </file>
@@ -751,10 +758,10 @@
         <v>14</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -762,10 +769,10 @@
         <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -773,10 +780,10 @@
         <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -784,10 +791,10 @@
         <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -795,10 +802,10 @@
         <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -806,10 +813,10 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -842,10 +849,10 @@
         <v>14</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -853,10 +860,10 @@
         <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -864,10 +871,10 @@
         <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -875,10 +882,10 @@
         <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -886,10 +893,10 @@
         <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -897,10 +904,10 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -970,7 +977,7 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>76</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>15</v>
@@ -981,7 +988,7 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>77</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>17</v>
@@ -992,7 +999,7 @@
         <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>78</v>
       </c>
       <c r="C4" s="4">
         <v>3</v>
@@ -1003,7 +1010,7 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>79</v>
       </c>
       <c r="C5" s="4">
         <v>5</v>
@@ -1014,7 +1021,7 @@
         <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="C6" s="4">
         <v>-2</v>
@@ -1025,10 +1032,10 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1083,7 +1090,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C4" s="4">
         <v>-2</v>
@@ -1094,10 +1101,10 @@
         <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1131,10 +1138,10 @@
         <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D2" s="1"/>
     </row>
@@ -1143,10 +1150,10 @@
         <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D3" s="1"/>
     </row>
@@ -1155,7 +1162,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C4" s="1">
         <v>0</v>
@@ -1167,7 +1174,7 @@
         <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C5" s="1">
         <v>3650</v>
@@ -1179,10 +1186,10 @@
         <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D6" s="1"/>
     </row>
@@ -1191,10 +1198,10 @@
         <v>14</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D7" s="1"/>
     </row>
@@ -1203,10 +1210,10 @@
         <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D8" s="1"/>
     </row>
@@ -1215,10 +1222,10 @@
         <v>14</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D9" s="1"/>
     </row>
@@ -1264,10 +1271,10 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1275,7 +1282,7 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -1286,13 +1293,13 @@
         <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="M4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -1300,10 +1307,10 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -1311,10 +1318,10 @@
         <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -1322,10 +1329,10 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -1333,10 +1340,10 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -1344,10 +1351,10 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -1355,10 +1362,10 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -1366,10 +1373,10 @@
         <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -1377,10 +1384,10 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -1388,10 +1395,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1423,10 +1430,10 @@
         <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1434,10 +1441,10 @@
         <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1445,7 +1452,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C4" s="1">
         <v>0</v>
@@ -1456,7 +1463,7 @@
         <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C5" s="1">
         <v>3650</v>
@@ -1467,10 +1474,10 @@
         <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1478,10 +1485,10 @@
         <v>14</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1489,10 +1496,10 @@
         <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1500,10 +1507,10 @@
         <v>14</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1536,10 +1543,10 @@
         <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1547,10 +1554,10 @@
         <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1558,7 +1565,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C4" s="1">
         <v>0</v>
@@ -1569,7 +1576,7 @@
         <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C5" s="1">
         <v>3650</v>
@@ -1580,10 +1587,10 @@
         <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1591,10 +1598,10 @@
         <v>14</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1602,10 +1609,10 @@
         <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1613,10 +1620,10 @@
         <v>14</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1661,7 +1668,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>5</v>
@@ -1969,10 +1976,10 @@
         <v>14</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1980,10 +1987,10 @@
         <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1991,10 +1998,10 @@
         <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2002,10 +2009,10 @@
         <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2013,10 +2020,10 @@
         <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2024,10 +2031,10 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -2061,10 +2068,10 @@
         <v>14</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2072,10 +2079,10 @@
         <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2083,10 +2090,10 @@
         <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2094,10 +2101,10 @@
         <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2105,10 +2112,10 @@
         <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2116,10 +2123,10 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2152,10 +2159,10 @@
         <v>14</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2163,10 +2170,10 @@
         <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2174,10 +2181,10 @@
         <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2185,10 +2192,10 @@
         <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2196,10 +2203,10 @@
         <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2207,10 +2214,10 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>